<commit_message>
MITRE plan phase A6: customer template upgrade + optional health columns (migration 036)
</commit_message>
<xml_diff>
--- a/apps/web/public/templates/scopewise-mitre-environment.xlsx
+++ b/apps/web/public/templates/scopewise-mitre-environment.xlsx
@@ -7,10 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Log Sources" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Tooling" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crown Jewels" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read Me" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Assets" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Log Sources" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Security Tooling" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Crown Jewels" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="2">
+  <fonts count="5">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -30,6 +31,17 @@
     </font>
     <font>
       <b val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <sz val="11"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="2">
@@ -52,9 +64,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -420,51 +441,77 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="100" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Platform</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>Windows</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>Linux</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>Azure AD</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>AWS</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>Microsoft 365</t>
+    <row r="1" ht="30" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>ScopeWise MITRE Environment Workbook</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="8" customHeight="1">
+      <c r="A2" s="3" t="n"/>
+    </row>
+    <row r="3" ht="30" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>This workbook is optional. Uploading it lets ScopeWise filter out techniques that don't apply to your environment and prioritize gaps by what you could realistically detect first. Skipping it still produces a coverage assessment -- just a conservative lower bound.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="8" customHeight="1">
+      <c r="A4" s="3" t="n"/>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Sheets in this workbook (all optional -- a missing sheet is noted as an assumption, never an error):</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="8" customHeight="1">
+      <c r="A6" s="3" t="n"/>
+    </row>
+    <row r="7" ht="30" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Assets -- your platform/technology inventory (e.g. Windows, AWS, Azure AD). Used to mark techniques that don't apply to any platform you have (e.g. macOS-only techniques when you have no Mac fleet) as Not Applicable.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Log Sources -- telemetry you already collect (e.g. Sysmon, CloudTrail). Used to prioritize gaps you could detect right now with data you already have. Optional health columns (Parser / Format, Normalized (Y/N), Last Event Seen) sharpen that prioritization -- a source that isn't normalized or hasn't seen recent events is treated as needing attention before you rely on it, not as fully ready.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Security Tooling -- products you own but may not have onboarded for logging yet. Used for the next-tier "onboard this, then detect" gaps.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Crown Jewels -- free text describing your most critical assets (e.g. "customer database", "payment gateway"). Used only to nudge the order gaps are shown in when they're relevant to what you described -- it never changes a coverage percentage or a technique's status.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="8" customHeight="1">
+      <c r="A11" s="3" t="n"/>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Honesty note: ScopeWise never ingests raw logs and never verifies a specific field is present in your data. Everything here is metadata you tell us about your environment -- if something looks off, it's worth double-checking your own inventory, not just trusting this workbook.</t>
         </is>
       </c>
     </row>
@@ -479,7 +526,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A4"/>
+  <dimension ref="A1:A6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -488,28 +535,42 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Source</t>
+          <t>Platform</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Sysmon</t>
+          <t>Windows</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Windows Event Logs</t>
+          <t>Linux</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CloudTrail</t>
+          <t>Azure AD</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>AWS</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Microsoft 365</t>
         </is>
       </c>
     </row>
@@ -524,30 +585,106 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Tool</t>
+          <t>Source</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Present?</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Parser / Format</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Normalized (Y/N)</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Last Event Seen</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>CrowdStrike Falcon EDR</t>
+          <t>Sysmon</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Sysmon XML</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>2026-08-01</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Proofpoint Email Security</t>
+          <t>Windows Event Logs</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>CloudTrail</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>CloudTrail JSON</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>2025-03-15</t>
         </is>
       </c>
     </row>
@@ -571,6 +708,44 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Tool</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>CrowdStrike Falcon EDR</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Proofpoint Email Security</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="30" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
           <t>Asset</t>
         </is>
       </c>

</xml_diff>

<commit_message>
MITRE A10 piece 2: one-row-per-log-stream guidance
Environment template's Read Me sheet gains one plain line (values-only
openpyxl edit, sheet names/headers byte-identical) plus a matching line
in the wizard's environment drop-zone: if one device sends more than one
kind of log, list each log type as its own row (e.g. 'Infoblox - DNS
logs' and 'Infoblox - SSH logs') so each stream gets credited
separately.
</commit_message>
<xml_diff>
--- a/apps/web/public/templates/scopewise-mitre-environment.xlsx
+++ b/apps/web/public/templates/scopewise-mitre-environment.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A12"/>
+  <dimension ref="A1:A13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -494,22 +494,29 @@
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Security Tooling -- products you own but may not have onboarded for logging yet. Used for the next-tier "onboard this, then detect" gaps.</t>
+          <t>Tip: if one device sends more than one kind of log, list each log type as its own row in Log Sources -- e.g. "Infoblox - DNS logs" and "Infoblox - SSH logs" -- so each stream gets credited separately.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="3" t="inlineStr">
         <is>
+          <t>Security Tooling -- products you own but may not have onboarded for logging yet. Used for the next-tier "onboard this, then detect" gaps.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="8" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
           <t>Crown Jewels -- free text describing your most critical assets (e.g. "customer database", "payment gateway"). Used only to nudge the order gaps are shown in when they're relevant to what you described -- it never changes a coverage percentage or a technique's status.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="8" customHeight="1">
-      <c r="A11" s="3" t="n"/>
-    </row>
     <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="3" t="inlineStr">
+      <c r="A12" s="3" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Honesty note: ScopeWise never ingests raw logs and never verifies a specific field is present in your data. Everything here is metadata you tell us about your environment -- if something looks off, it's worth double-checking your own inventory, not just trusting this workbook.</t>
         </is>

</xml_diff>

<commit_message>
MITRE A11 piece 2: regenerate templates with styling
New committed scripts/build_mitre_templates.py generator (prefer this
over hand-editing the templates going forward). Both downloadable
templates regenerated: branded header fill + white bold font (same
family as the XLSX report), thin all-borders on header + example rows,
~100 pre-formatted blank data rows per sheet so entered content lands in
a visible grid, sized column widths. All cell VALUES verified
byte-identical to what shipped before (diffed cell-by-cell against git
HEAD, ignoring the new trailing blank rows); the existing ingest
round-trip tests pass unchanged. Side fix: the environment template's
Read Me sheet had two swapped row heights and one row with no explicit
height at all, left over from an earlier ad hoc insert_rows() edit --
the generator sets every row height explicitly, correctly, now. New
readback test checks header fill/font/border and blank-row count for
both templates.
</commit_message>
<xml_diff>
--- a/apps/web/public/templates/scopewise-mitre-environment.xlsx
+++ b/apps/web/public/templates/scopewise-mitre-environment.xlsx
@@ -21,7 +21,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -31,28 +31,37 @@
     </font>
     <font>
       <b val="1"/>
+      <sz val="14"/>
+    </font>
+    <font/>
+    <font>
+      <b val="1"/>
     </font>
     <font>
       <b val="1"/>
+      <color rgb="00FFFFFF"/>
       <sz val="14"/>
     </font>
     <font>
-      <sz val="11"/>
-    </font>
-    <font>
       <b val="1"/>
-      <sz val="11"/>
+      <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="000057B8"/>
+        <bgColor rgb="000057B8"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -60,22 +69,42 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="008496AD"/>
+      </left>
+      <right style="thin">
+        <color rgb="008496AD"/>
+      </right>
+      <top style="thin">
+        <color rgb="008496AD"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="008496AD"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -448,75 +477,75 @@
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>ScopeWise MITRE Environment Workbook</t>
         </is>
       </c>
     </row>
     <row r="2" ht="8" customHeight="1">
-      <c r="A2" s="3" t="n"/>
+      <c r="A2" s="2" t="n"/>
     </row>
     <row r="3" ht="30" customHeight="1">
-      <c r="A3" s="3" t="inlineStr">
+      <c r="A3" s="2" t="inlineStr">
         <is>
           <t>This workbook is optional. Uploading it lets ScopeWise filter out techniques that don't apply to your environment and prioritize gaps by what you could realistically detect first. Skipping it still produces a coverage assessment -- just a conservative lower bound.</t>
         </is>
       </c>
     </row>
     <row r="4" ht="8" customHeight="1">
-      <c r="A4" s="3" t="n"/>
+      <c r="A4" s="2" t="n"/>
     </row>
     <row r="5" ht="30" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t>Sheets in this workbook (all optional -- a missing sheet is noted as an assumption, never an error):</t>
         </is>
       </c>
     </row>
     <row r="6" ht="8" customHeight="1">
-      <c r="A6" s="3" t="n"/>
+      <c r="A6" s="2" t="n"/>
     </row>
     <row r="7" ht="30" customHeight="1">
-      <c r="A7" s="3" t="inlineStr">
+      <c r="A7" s="2" t="inlineStr">
         <is>
           <t>Assets -- your platform/technology inventory (e.g. Windows, AWS, Azure AD). Used to mark techniques that don't apply to any platform you have (e.g. macOS-only techniques when you have no Mac fleet) as Not Applicable.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
-      <c r="A8" s="3" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>Log Sources -- telemetry you already collect (e.g. Sysmon, CloudTrail). Used to prioritize gaps you could detect right now with data you already have. Optional health columns (Parser / Format, Normalized (Y/N), Last Event Seen) sharpen that prioritization -- a source that isn't normalized or hasn't seen recent events is treated as needing attention before you rely on it, not as fully ready.</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="3" t="inlineStr">
+      <c r="A9" s="2" t="inlineStr">
         <is>
           <t>Tip: if one device sends more than one kind of log, list each log type as its own row in Log Sources -- e.g. "Infoblox - DNS logs" and "Infoblox - SSH logs" -- so each stream gets credited separately.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="3" t="inlineStr">
+      <c r="A10" s="2" t="inlineStr">
         <is>
           <t>Security Tooling -- products you own but may not have onboarded for logging yet. Used for the next-tier "onboard this, then detect" gaps.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="8" customHeight="1">
-      <c r="A11" s="3" t="inlineStr">
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="2" t="inlineStr">
         <is>
           <t>Crown Jewels -- free text describing your most critical assets (e.g. "customer database", "payment gateway"). Used only to nudge the order gaps are shown in when they're relevant to what you described -- it never changes a coverage percentage or a technique's status.</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="30" customHeight="1">
-      <c r="A12" s="3" t="n"/>
-    </row>
-    <row r="13">
-      <c r="A13" s="3" t="inlineStr">
+    <row r="12" ht="8" customHeight="1">
+      <c r="A12" s="2" t="n"/>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="2" t="inlineStr">
         <is>
           <t>Honesty note: ScopeWise never ingests raw logs and never verifies a specific field is present in your data. Everything here is metadata you tell us about your environment -- if something looks off, it's worth double-checking your own inventory, not just trusting this workbook.</t>
         </is>
@@ -533,53 +562,353 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A106"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Platform</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>Windows</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>Linux</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Azure AD</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>AWS</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" s="5" t="inlineStr">
         <is>
           <t>Microsoft 365</t>
         </is>
       </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="6" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="6" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="6" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="6" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="6" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="6" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="6" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="6" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="6" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="6" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="6" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="6" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="6" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="6" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="6" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="6" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="6" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="6" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="6" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="6" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="6" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="6" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="6" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="6" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="6" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="6" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="6" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="6" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="6" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="6" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="6" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="6" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="6" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="6" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="6" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="6" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="6" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="6" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="6" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="6" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="6" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="6" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="6" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="6" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="6" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="6" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="6" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="6" t="n"/>
+    </row>
+    <row r="105">
+      <c r="A105" s="6" t="n"/>
+    </row>
+    <row r="106">
+      <c r="A106" s="6" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -592,7 +921,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E104"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -603,97 +932,800 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>Present?</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>Parser / Format</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="4" t="inlineStr">
         <is>
           <t>Normalized (Y/N)</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="4" t="inlineStr">
         <is>
           <t>Last Event Seen</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>Sysmon</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="B2" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr">
+      <c r="C2" s="5" t="inlineStr">
         <is>
           <t>Sysmon XML</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr">
+      <c r="D2" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="5" t="inlineStr">
         <is>
           <t>2026-08-01</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>Windows Event Logs</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="B3" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
+      <c r="C3" s="5" t="n"/>
+      <c r="D3" s="5" t="n"/>
+      <c r="E3" s="5" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>CloudTrail</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="B4" s="5" t="inlineStr">
         <is>
           <t>Yes</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr">
+      <c r="C4" s="5" t="inlineStr">
         <is>
           <t>CloudTrail JSON</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr">
+      <c r="D4" s="5" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="E4" s="5" t="inlineStr">
         <is>
           <t>2025-03-15</t>
         </is>
       </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="n"/>
+      <c r="B5" s="6" t="n"/>
+      <c r="C5" s="6" t="n"/>
+      <c r="D5" s="6" t="n"/>
+      <c r="E5" s="6" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="n"/>
+      <c r="B6" s="6" t="n"/>
+      <c r="C6" s="6" t="n"/>
+      <c r="D6" s="6" t="n"/>
+      <c r="E6" s="6" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="n"/>
+      <c r="B7" s="6" t="n"/>
+      <c r="C7" s="6" t="n"/>
+      <c r="D7" s="6" t="n"/>
+      <c r="E7" s="6" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="n"/>
+      <c r="B8" s="6" t="n"/>
+      <c r="C8" s="6" t="n"/>
+      <c r="D8" s="6" t="n"/>
+      <c r="E8" s="6" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="n"/>
+      <c r="B9" s="6" t="n"/>
+      <c r="C9" s="6" t="n"/>
+      <c r="D9" s="6" t="n"/>
+      <c r="E9" s="6" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="n"/>
+      <c r="B10" s="6" t="n"/>
+      <c r="C10" s="6" t="n"/>
+      <c r="D10" s="6" t="n"/>
+      <c r="E10" s="6" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n"/>
+      <c r="B11" s="6" t="n"/>
+      <c r="C11" s="6" t="n"/>
+      <c r="D11" s="6" t="n"/>
+      <c r="E11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n"/>
+      <c r="B12" s="6" t="n"/>
+      <c r="C12" s="6" t="n"/>
+      <c r="D12" s="6" t="n"/>
+      <c r="E12" s="6" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="n"/>
+      <c r="B13" s="6" t="n"/>
+      <c r="C13" s="6" t="n"/>
+      <c r="D13" s="6" t="n"/>
+      <c r="E13" s="6" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="n"/>
+      <c r="B14" s="6" t="n"/>
+      <c r="C14" s="6" t="n"/>
+      <c r="D14" s="6" t="n"/>
+      <c r="E14" s="6" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="n"/>
+      <c r="B15" s="6" t="n"/>
+      <c r="C15" s="6" t="n"/>
+      <c r="D15" s="6" t="n"/>
+      <c r="E15" s="6" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="n"/>
+      <c r="B16" s="6" t="n"/>
+      <c r="C16" s="6" t="n"/>
+      <c r="D16" s="6" t="n"/>
+      <c r="E16" s="6" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="n"/>
+      <c r="B17" s="6" t="n"/>
+      <c r="C17" s="6" t="n"/>
+      <c r="D17" s="6" t="n"/>
+      <c r="E17" s="6" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="n"/>
+      <c r="B18" s="6" t="n"/>
+      <c r="C18" s="6" t="n"/>
+      <c r="D18" s="6" t="n"/>
+      <c r="E18" s="6" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="n"/>
+      <c r="B19" s="6" t="n"/>
+      <c r="C19" s="6" t="n"/>
+      <c r="D19" s="6" t="n"/>
+      <c r="E19" s="6" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="n"/>
+      <c r="B20" s="6" t="n"/>
+      <c r="C20" s="6" t="n"/>
+      <c r="D20" s="6" t="n"/>
+      <c r="E20" s="6" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="n"/>
+      <c r="B21" s="6" t="n"/>
+      <c r="C21" s="6" t="n"/>
+      <c r="D21" s="6" t="n"/>
+      <c r="E21" s="6" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="n"/>
+      <c r="B22" s="6" t="n"/>
+      <c r="C22" s="6" t="n"/>
+      <c r="D22" s="6" t="n"/>
+      <c r="E22" s="6" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="n"/>
+      <c r="B23" s="6" t="n"/>
+      <c r="C23" s="6" t="n"/>
+      <c r="D23" s="6" t="n"/>
+      <c r="E23" s="6" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="n"/>
+      <c r="B24" s="6" t="n"/>
+      <c r="C24" s="6" t="n"/>
+      <c r="D24" s="6" t="n"/>
+      <c r="E24" s="6" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="n"/>
+      <c r="B25" s="6" t="n"/>
+      <c r="C25" s="6" t="n"/>
+      <c r="D25" s="6" t="n"/>
+      <c r="E25" s="6" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="n"/>
+      <c r="B26" s="6" t="n"/>
+      <c r="C26" s="6" t="n"/>
+      <c r="D26" s="6" t="n"/>
+      <c r="E26" s="6" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="n"/>
+      <c r="B27" s="6" t="n"/>
+      <c r="C27" s="6" t="n"/>
+      <c r="D27" s="6" t="n"/>
+      <c r="E27" s="6" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="n"/>
+      <c r="B28" s="6" t="n"/>
+      <c r="C28" s="6" t="n"/>
+      <c r="D28" s="6" t="n"/>
+      <c r="E28" s="6" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="n"/>
+      <c r="B29" s="6" t="n"/>
+      <c r="C29" s="6" t="n"/>
+      <c r="D29" s="6" t="n"/>
+      <c r="E29" s="6" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="n"/>
+      <c r="B30" s="6" t="n"/>
+      <c r="C30" s="6" t="n"/>
+      <c r="D30" s="6" t="n"/>
+      <c r="E30" s="6" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="n"/>
+      <c r="B31" s="6" t="n"/>
+      <c r="C31" s="6" t="n"/>
+      <c r="D31" s="6" t="n"/>
+      <c r="E31" s="6" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="n"/>
+      <c r="B32" s="6" t="n"/>
+      <c r="C32" s="6" t="n"/>
+      <c r="D32" s="6" t="n"/>
+      <c r="E32" s="6" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="n"/>
+      <c r="B33" s="6" t="n"/>
+      <c r="C33" s="6" t="n"/>
+      <c r="D33" s="6" t="n"/>
+      <c r="E33" s="6" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="n"/>
+      <c r="B34" s="6" t="n"/>
+      <c r="C34" s="6" t="n"/>
+      <c r="D34" s="6" t="n"/>
+      <c r="E34" s="6" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="n"/>
+      <c r="B35" s="6" t="n"/>
+      <c r="C35" s="6" t="n"/>
+      <c r="D35" s="6" t="n"/>
+      <c r="E35" s="6" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="n"/>
+      <c r="B36" s="6" t="n"/>
+      <c r="C36" s="6" t="n"/>
+      <c r="D36" s="6" t="n"/>
+      <c r="E36" s="6" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="n"/>
+      <c r="B37" s="6" t="n"/>
+      <c r="C37" s="6" t="n"/>
+      <c r="D37" s="6" t="n"/>
+      <c r="E37" s="6" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="n"/>
+      <c r="B38" s="6" t="n"/>
+      <c r="C38" s="6" t="n"/>
+      <c r="D38" s="6" t="n"/>
+      <c r="E38" s="6" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="n"/>
+      <c r="B39" s="6" t="n"/>
+      <c r="C39" s="6" t="n"/>
+      <c r="D39" s="6" t="n"/>
+      <c r="E39" s="6" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="n"/>
+      <c r="B40" s="6" t="n"/>
+      <c r="C40" s="6" t="n"/>
+      <c r="D40" s="6" t="n"/>
+      <c r="E40" s="6" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="n"/>
+      <c r="B41" s="6" t="n"/>
+      <c r="C41" s="6" t="n"/>
+      <c r="D41" s="6" t="n"/>
+      <c r="E41" s="6" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="n"/>
+      <c r="B42" s="6" t="n"/>
+      <c r="C42" s="6" t="n"/>
+      <c r="D42" s="6" t="n"/>
+      <c r="E42" s="6" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="n"/>
+      <c r="B43" s="6" t="n"/>
+      <c r="C43" s="6" t="n"/>
+      <c r="D43" s="6" t="n"/>
+      <c r="E43" s="6" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="n"/>
+      <c r="B44" s="6" t="n"/>
+      <c r="C44" s="6" t="n"/>
+      <c r="D44" s="6" t="n"/>
+      <c r="E44" s="6" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="n"/>
+      <c r="B45" s="6" t="n"/>
+      <c r="C45" s="6" t="n"/>
+      <c r="D45" s="6" t="n"/>
+      <c r="E45" s="6" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="n"/>
+      <c r="B46" s="6" t="n"/>
+      <c r="C46" s="6" t="n"/>
+      <c r="D46" s="6" t="n"/>
+      <c r="E46" s="6" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="n"/>
+      <c r="B47" s="6" t="n"/>
+      <c r="C47" s="6" t="n"/>
+      <c r="D47" s="6" t="n"/>
+      <c r="E47" s="6" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="n"/>
+      <c r="B48" s="6" t="n"/>
+      <c r="C48" s="6" t="n"/>
+      <c r="D48" s="6" t="n"/>
+      <c r="E48" s="6" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="n"/>
+      <c r="B49" s="6" t="n"/>
+      <c r="C49" s="6" t="n"/>
+      <c r="D49" s="6" t="n"/>
+      <c r="E49" s="6" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="n"/>
+      <c r="B50" s="6" t="n"/>
+      <c r="C50" s="6" t="n"/>
+      <c r="D50" s="6" t="n"/>
+      <c r="E50" s="6" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="n"/>
+      <c r="B51" s="6" t="n"/>
+      <c r="C51" s="6" t="n"/>
+      <c r="D51" s="6" t="n"/>
+      <c r="E51" s="6" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="n"/>
+      <c r="B52" s="6" t="n"/>
+      <c r="C52" s="6" t="n"/>
+      <c r="D52" s="6" t="n"/>
+      <c r="E52" s="6" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="6" t="n"/>
+      <c r="B53" s="6" t="n"/>
+      <c r="C53" s="6" t="n"/>
+      <c r="D53" s="6" t="n"/>
+      <c r="E53" s="6" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="n"/>
+      <c r="B54" s="6" t="n"/>
+      <c r="C54" s="6" t="n"/>
+      <c r="D54" s="6" t="n"/>
+      <c r="E54" s="6" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="n"/>
+      <c r="B55" s="6" t="n"/>
+      <c r="C55" s="6" t="n"/>
+      <c r="D55" s="6" t="n"/>
+      <c r="E55" s="6" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="6" t="n"/>
+      <c r="B56" s="6" t="n"/>
+      <c r="C56" s="6" t="n"/>
+      <c r="D56" s="6" t="n"/>
+      <c r="E56" s="6" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="6" t="n"/>
+      <c r="B57" s="6" t="n"/>
+      <c r="C57" s="6" t="n"/>
+      <c r="D57" s="6" t="n"/>
+      <c r="E57" s="6" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="n"/>
+      <c r="B58" s="6" t="n"/>
+      <c r="C58" s="6" t="n"/>
+      <c r="D58" s="6" t="n"/>
+      <c r="E58" s="6" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="n"/>
+      <c r="B59" s="6" t="n"/>
+      <c r="C59" s="6" t="n"/>
+      <c r="D59" s="6" t="n"/>
+      <c r="E59" s="6" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="6" t="n"/>
+      <c r="B60" s="6" t="n"/>
+      <c r="C60" s="6" t="n"/>
+      <c r="D60" s="6" t="n"/>
+      <c r="E60" s="6" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="6" t="n"/>
+      <c r="B61" s="6" t="n"/>
+      <c r="C61" s="6" t="n"/>
+      <c r="D61" s="6" t="n"/>
+      <c r="E61" s="6" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="6" t="n"/>
+      <c r="B62" s="6" t="n"/>
+      <c r="C62" s="6" t="n"/>
+      <c r="D62" s="6" t="n"/>
+      <c r="E62" s="6" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="6" t="n"/>
+      <c r="B63" s="6" t="n"/>
+      <c r="C63" s="6" t="n"/>
+      <c r="D63" s="6" t="n"/>
+      <c r="E63" s="6" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="6" t="n"/>
+      <c r="B64" s="6" t="n"/>
+      <c r="C64" s="6" t="n"/>
+      <c r="D64" s="6" t="n"/>
+      <c r="E64" s="6" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="6" t="n"/>
+      <c r="B65" s="6" t="n"/>
+      <c r="C65" s="6" t="n"/>
+      <c r="D65" s="6" t="n"/>
+      <c r="E65" s="6" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="6" t="n"/>
+      <c r="B66" s="6" t="n"/>
+      <c r="C66" s="6" t="n"/>
+      <c r="D66" s="6" t="n"/>
+      <c r="E66" s="6" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="6" t="n"/>
+      <c r="B67" s="6" t="n"/>
+      <c r="C67" s="6" t="n"/>
+      <c r="D67" s="6" t="n"/>
+      <c r="E67" s="6" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="6" t="n"/>
+      <c r="B68" s="6" t="n"/>
+      <c r="C68" s="6" t="n"/>
+      <c r="D68" s="6" t="n"/>
+      <c r="E68" s="6" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="6" t="n"/>
+      <c r="B69" s="6" t="n"/>
+      <c r="C69" s="6" t="n"/>
+      <c r="D69" s="6" t="n"/>
+      <c r="E69" s="6" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="6" t="n"/>
+      <c r="B70" s="6" t="n"/>
+      <c r="C70" s="6" t="n"/>
+      <c r="D70" s="6" t="n"/>
+      <c r="E70" s="6" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="6" t="n"/>
+      <c r="B71" s="6" t="n"/>
+      <c r="C71" s="6" t="n"/>
+      <c r="D71" s="6" t="n"/>
+      <c r="E71" s="6" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="6" t="n"/>
+      <c r="B72" s="6" t="n"/>
+      <c r="C72" s="6" t="n"/>
+      <c r="D72" s="6" t="n"/>
+      <c r="E72" s="6" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="6" t="n"/>
+      <c r="B73" s="6" t="n"/>
+      <c r="C73" s="6" t="n"/>
+      <c r="D73" s="6" t="n"/>
+      <c r="E73" s="6" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="6" t="n"/>
+      <c r="B74" s="6" t="n"/>
+      <c r="C74" s="6" t="n"/>
+      <c r="D74" s="6" t="n"/>
+      <c r="E74" s="6" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="6" t="n"/>
+      <c r="B75" s="6" t="n"/>
+      <c r="C75" s="6" t="n"/>
+      <c r="D75" s="6" t="n"/>
+      <c r="E75" s="6" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="6" t="n"/>
+      <c r="B76" s="6" t="n"/>
+      <c r="C76" s="6" t="n"/>
+      <c r="D76" s="6" t="n"/>
+      <c r="E76" s="6" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="6" t="n"/>
+      <c r="B77" s="6" t="n"/>
+      <c r="C77" s="6" t="n"/>
+      <c r="D77" s="6" t="n"/>
+      <c r="E77" s="6" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="6" t="n"/>
+      <c r="B78" s="6" t="n"/>
+      <c r="C78" s="6" t="n"/>
+      <c r="D78" s="6" t="n"/>
+      <c r="E78" s="6" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="6" t="n"/>
+      <c r="B79" s="6" t="n"/>
+      <c r="C79" s="6" t="n"/>
+      <c r="D79" s="6" t="n"/>
+      <c r="E79" s="6" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="6" t="n"/>
+      <c r="B80" s="6" t="n"/>
+      <c r="C80" s="6" t="n"/>
+      <c r="D80" s="6" t="n"/>
+      <c r="E80" s="6" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="6" t="n"/>
+      <c r="B81" s="6" t="n"/>
+      <c r="C81" s="6" t="n"/>
+      <c r="D81" s="6" t="n"/>
+      <c r="E81" s="6" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="6" t="n"/>
+      <c r="B82" s="6" t="n"/>
+      <c r="C82" s="6" t="n"/>
+      <c r="D82" s="6" t="n"/>
+      <c r="E82" s="6" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="6" t="n"/>
+      <c r="B83" s="6" t="n"/>
+      <c r="C83" s="6" t="n"/>
+      <c r="D83" s="6" t="n"/>
+      <c r="E83" s="6" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="6" t="n"/>
+      <c r="B84" s="6" t="n"/>
+      <c r="C84" s="6" t="n"/>
+      <c r="D84" s="6" t="n"/>
+      <c r="E84" s="6" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="6" t="n"/>
+      <c r="B85" s="6" t="n"/>
+      <c r="C85" s="6" t="n"/>
+      <c r="D85" s="6" t="n"/>
+      <c r="E85" s="6" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="6" t="n"/>
+      <c r="B86" s="6" t="n"/>
+      <c r="C86" s="6" t="n"/>
+      <c r="D86" s="6" t="n"/>
+      <c r="E86" s="6" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="6" t="n"/>
+      <c r="B87" s="6" t="n"/>
+      <c r="C87" s="6" t="n"/>
+      <c r="D87" s="6" t="n"/>
+      <c r="E87" s="6" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="6" t="n"/>
+      <c r="B88" s="6" t="n"/>
+      <c r="C88" s="6" t="n"/>
+      <c r="D88" s="6" t="n"/>
+      <c r="E88" s="6" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="6" t="n"/>
+      <c r="B89" s="6" t="n"/>
+      <c r="C89" s="6" t="n"/>
+      <c r="D89" s="6" t="n"/>
+      <c r="E89" s="6" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="6" t="n"/>
+      <c r="B90" s="6" t="n"/>
+      <c r="C90" s="6" t="n"/>
+      <c r="D90" s="6" t="n"/>
+      <c r="E90" s="6" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="6" t="n"/>
+      <c r="B91" s="6" t="n"/>
+      <c r="C91" s="6" t="n"/>
+      <c r="D91" s="6" t="n"/>
+      <c r="E91" s="6" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="6" t="n"/>
+      <c r="B92" s="6" t="n"/>
+      <c r="C92" s="6" t="n"/>
+      <c r="D92" s="6" t="n"/>
+      <c r="E92" s="6" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="6" t="n"/>
+      <c r="B93" s="6" t="n"/>
+      <c r="C93" s="6" t="n"/>
+      <c r="D93" s="6" t="n"/>
+      <c r="E93" s="6" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="6" t="n"/>
+      <c r="B94" s="6" t="n"/>
+      <c r="C94" s="6" t="n"/>
+      <c r="D94" s="6" t="n"/>
+      <c r="E94" s="6" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="6" t="n"/>
+      <c r="B95" s="6" t="n"/>
+      <c r="C95" s="6" t="n"/>
+      <c r="D95" s="6" t="n"/>
+      <c r="E95" s="6" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="6" t="n"/>
+      <c r="B96" s="6" t="n"/>
+      <c r="C96" s="6" t="n"/>
+      <c r="D96" s="6" t="n"/>
+      <c r="E96" s="6" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="6" t="n"/>
+      <c r="B97" s="6" t="n"/>
+      <c r="C97" s="6" t="n"/>
+      <c r="D97" s="6" t="n"/>
+      <c r="E97" s="6" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="6" t="n"/>
+      <c r="B98" s="6" t="n"/>
+      <c r="C98" s="6" t="n"/>
+      <c r="D98" s="6" t="n"/>
+      <c r="E98" s="6" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="6" t="n"/>
+      <c r="B99" s="6" t="n"/>
+      <c r="C99" s="6" t="n"/>
+      <c r="D99" s="6" t="n"/>
+      <c r="E99" s="6" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="6" t="n"/>
+      <c r="B100" s="6" t="n"/>
+      <c r="C100" s="6" t="n"/>
+      <c r="D100" s="6" t="n"/>
+      <c r="E100" s="6" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="6" t="n"/>
+      <c r="B101" s="6" t="n"/>
+      <c r="C101" s="6" t="n"/>
+      <c r="D101" s="6" t="n"/>
+      <c r="E101" s="6" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="6" t="n"/>
+      <c r="B102" s="6" t="n"/>
+      <c r="C102" s="6" t="n"/>
+      <c r="D102" s="6" t="n"/>
+      <c r="E102" s="6" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="6" t="n"/>
+      <c r="B103" s="6" t="n"/>
+      <c r="C103" s="6" t="n"/>
+      <c r="D103" s="6" t="n"/>
+      <c r="E103" s="6" t="n"/>
+    </row>
+    <row r="104">
+      <c r="A104" s="6" t="n"/>
+      <c r="B104" s="6" t="n"/>
+      <c r="C104" s="6" t="n"/>
+      <c r="D104" s="6" t="n"/>
+      <c r="E104" s="6" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -706,32 +1738,332 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:A103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Tool</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>CrowdStrike Falcon EDR</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>Proofpoint Email Security</t>
         </is>
       </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="6" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="6" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="6" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="6" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="6" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="6" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="6" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="6" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="6" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="6" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="6" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="6" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="6" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="6" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="6" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="6" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="6" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="6" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="6" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="6" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="6" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="6" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="6" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="6" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="6" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="6" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="6" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="6" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="6" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="6" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="6" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="6" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="6" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="6" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="6" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="6" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="6" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="6" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="6" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="6" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="6" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="6" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="6" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="6" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="6" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="6" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="6" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -744,32 +2076,332 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A3"/>
+  <dimension ref="A1:A103"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Asset</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="5" t="inlineStr">
         <is>
           <t>Customer database</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" s="5" t="inlineStr">
         <is>
           <t>Payment processing service</t>
         </is>
       </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="6" t="n"/>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="n"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="6" t="n"/>
+    </row>
+    <row r="7">
+      <c r="A7" s="6" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="6" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="6" t="n"/>
+    </row>
+    <row r="10">
+      <c r="A10" s="6" t="n"/>
+    </row>
+    <row r="11">
+      <c r="A11" s="6" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="6" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="6" t="n"/>
+    </row>
+    <row r="14">
+      <c r="A14" s="6" t="n"/>
+    </row>
+    <row r="15">
+      <c r="A15" s="6" t="n"/>
+    </row>
+    <row r="16">
+      <c r="A16" s="6" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="6" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="6" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="6" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="6" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="6" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="6" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="6" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="6" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="6" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="6" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="6" t="n"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="6" t="n"/>
+    </row>
+    <row r="29">
+      <c r="A29" s="6" t="n"/>
+    </row>
+    <row r="30">
+      <c r="A30" s="6" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="6" t="n"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="6" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="6" t="n"/>
+    </row>
+    <row r="34">
+      <c r="A34" s="6" t="n"/>
+    </row>
+    <row r="35">
+      <c r="A35" s="6" t="n"/>
+    </row>
+    <row r="36">
+      <c r="A36" s="6" t="n"/>
+    </row>
+    <row r="37">
+      <c r="A37" s="6" t="n"/>
+    </row>
+    <row r="38">
+      <c r="A38" s="6" t="n"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="n"/>
+    </row>
+    <row r="40">
+      <c r="A40" s="6" t="n"/>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="n"/>
+    </row>
+    <row r="42">
+      <c r="A42" s="6" t="n"/>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="n"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="6" t="n"/>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="n"/>
+    </row>
+    <row r="46">
+      <c r="A46" s="6" t="n"/>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="n"/>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="n"/>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="n"/>
+    </row>
+    <row r="50">
+      <c r="A50" s="6" t="n"/>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="n"/>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="n"/>
+    </row>
+    <row r="53">
+      <c r="A53" s="6" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="n"/>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="n"/>
+    </row>
+    <row r="56">
+      <c r="A56" s="6" t="n"/>
+    </row>
+    <row r="57">
+      <c r="A57" s="6" t="n"/>
+    </row>
+    <row r="58">
+      <c r="A58" s="6" t="n"/>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="n"/>
+    </row>
+    <row r="60">
+      <c r="A60" s="6" t="n"/>
+    </row>
+    <row r="61">
+      <c r="A61" s="6" t="n"/>
+    </row>
+    <row r="62">
+      <c r="A62" s="6" t="n"/>
+    </row>
+    <row r="63">
+      <c r="A63" s="6" t="n"/>
+    </row>
+    <row r="64">
+      <c r="A64" s="6" t="n"/>
+    </row>
+    <row r="65">
+      <c r="A65" s="6" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" s="6" t="n"/>
+    </row>
+    <row r="67">
+      <c r="A67" s="6" t="n"/>
+    </row>
+    <row r="68">
+      <c r="A68" s="6" t="n"/>
+    </row>
+    <row r="69">
+      <c r="A69" s="6" t="n"/>
+    </row>
+    <row r="70">
+      <c r="A70" s="6" t="n"/>
+    </row>
+    <row r="71">
+      <c r="A71" s="6" t="n"/>
+    </row>
+    <row r="72">
+      <c r="A72" s="6" t="n"/>
+    </row>
+    <row r="73">
+      <c r="A73" s="6" t="n"/>
+    </row>
+    <row r="74">
+      <c r="A74" s="6" t="n"/>
+    </row>
+    <row r="75">
+      <c r="A75" s="6" t="n"/>
+    </row>
+    <row r="76">
+      <c r="A76" s="6" t="n"/>
+    </row>
+    <row r="77">
+      <c r="A77" s="6" t="n"/>
+    </row>
+    <row r="78">
+      <c r="A78" s="6" t="n"/>
+    </row>
+    <row r="79">
+      <c r="A79" s="6" t="n"/>
+    </row>
+    <row r="80">
+      <c r="A80" s="6" t="n"/>
+    </row>
+    <row r="81">
+      <c r="A81" s="6" t="n"/>
+    </row>
+    <row r="82">
+      <c r="A82" s="6" t="n"/>
+    </row>
+    <row r="83">
+      <c r="A83" s="6" t="n"/>
+    </row>
+    <row r="84">
+      <c r="A84" s="6" t="n"/>
+    </row>
+    <row r="85">
+      <c r="A85" s="6" t="n"/>
+    </row>
+    <row r="86">
+      <c r="A86" s="6" t="n"/>
+    </row>
+    <row r="87">
+      <c r="A87" s="6" t="n"/>
+    </row>
+    <row r="88">
+      <c r="A88" s="6" t="n"/>
+    </row>
+    <row r="89">
+      <c r="A89" s="6" t="n"/>
+    </row>
+    <row r="90">
+      <c r="A90" s="6" t="n"/>
+    </row>
+    <row r="91">
+      <c r="A91" s="6" t="n"/>
+    </row>
+    <row r="92">
+      <c r="A92" s="6" t="n"/>
+    </row>
+    <row r="93">
+      <c r="A93" s="6" t="n"/>
+    </row>
+    <row r="94">
+      <c r="A94" s="6" t="n"/>
+    </row>
+    <row r="95">
+      <c r="A95" s="6" t="n"/>
+    </row>
+    <row r="96">
+      <c r="A96" s="6" t="n"/>
+    </row>
+    <row r="97">
+      <c r="A97" s="6" t="n"/>
+    </row>
+    <row r="98">
+      <c r="A98" s="6" t="n"/>
+    </row>
+    <row r="99">
+      <c r="A99" s="6" t="n"/>
+    </row>
+    <row r="100">
+      <c r="A100" s="6" t="n"/>
+    </row>
+    <row r="101">
+      <c r="A101" s="6" t="n"/>
+    </row>
+    <row r="102">
+      <c r="A102" s="6" t="n"/>
+    </row>
+    <row r="103">
+      <c r="A103" s="6" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>